<commit_message>
Ajout du projet Tasty Crousty V2 dans E5
</commit_message>
<xml_diff>
--- a/e5/tableau_competences.xlsx
+++ b/e5/tableau_competences.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Autres ordinateurs\Mon ordinateur portable\Documents\PORTEFOLIO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e2f25182b63ad68a/Documents/PORTEFOLIO/e5/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3838D20B-7E0C-4472-B70D-4C76E24118F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4AF58D0-E6C5-40B8-A23E-99B808EF88C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$20</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -160,15 +160,6 @@
   <si>
     <t>Développement de l'employabilité et du réseau via Linkedin</t>
   </si>
-  <si>
-    <t>Simulation d'une infrastructure réseau d'entreprise avec segmentation VLAN, firewall pfSense et Active Directory</t>
-  </si>
-  <si>
-    <t>Procédure dotation d'un nouveau PC</t>
-  </si>
-  <si>
-    <t>Projet Etherchannel HSRP</t>
-  </si>
 </sst>
 </file>
 
@@ -177,7 +168,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -247,12 +238,6 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <sz val="8"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -537,7 +522,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -673,27 +658,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1004,17 +968,17 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ86"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:AQ84"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.42578125" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.42578125" customWidth="1"/>
-    <col min="44" max="16384" width="10.7109375" style="1"/>
+    <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.44140625" style="1" customWidth="1"/>
+    <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.44140625" customWidth="1"/>
+    <col min="44" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:43" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
@@ -1028,7 +992,7 @@
       </c>
       <c r="H1" s="38"/>
     </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
         <v>1</v>
       </c>
@@ -1040,7 +1004,7 @@
       <c r="G2" s="38"/>
       <c r="H2" s="38"/>
     </row>
-    <row r="3" spans="1:43" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:43" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="39" t="s">
         <v>28</v>
       </c>
@@ -1055,7 +1019,7 @@
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:43" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
         <v>2</v>
       </c>
@@ -1073,7 +1037,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:43" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="44" t="s">
         <v>31</v>
       </c>
@@ -1085,7 +1049,7 @@
       <c r="G5" s="45"/>
       <c r="H5" s="45"/>
     </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="42" t="s">
         <v>6</v>
       </c>
@@ -1111,7 +1075,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="325.14999999999998" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="325.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="43"/>
       <c r="B7" s="37"/>
       <c r="C7" s="19" t="s">
@@ -1168,7 +1132,7 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
         <v>20</v>
       </c>
@@ -1215,7 +1179,7 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>23</v>
       </c>
@@ -1264,7 +1228,7 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>24</v>
       </c>
@@ -1313,7 +1277,7 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>32</v>
       </c>
@@ -1362,19 +1326,19 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="46">
-        <v>46082</v>
-      </c>
-      <c r="C12" s="50"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="48"/>
-      <c r="F12" s="50"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="49"/>
+        <v>29</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="26"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1411,19 +1375,17 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="51">
-        <v>46029</v>
-      </c>
-      <c r="C13" s="50"/>
-      <c r="D13" s="50"/>
-      <c r="E13" s="48"/>
-      <c r="F13" s="50"/>
-      <c r="G13" s="50"/>
-      <c r="H13" s="49"/>
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="32"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1460,19 +1422,15 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="26"/>
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1509,17 +1467,15 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="31"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="32"/>
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1556,15 +1512,17 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="5"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="33" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="35"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1601,14 +1559,18 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="5"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="10"/>
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="21">
+        <v>45999</v>
+      </c>
+      <c r="C17" s="11"/>
+      <c r="D17" s="23"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="11"/>
       <c r="H17" s="10"/>
       <c r="I17"/>
       <c r="J17"/>
@@ -1646,17 +1608,19 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" s="34"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="35"/>
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="21">
+        <v>45988</v>
+      </c>
+      <c r="C18" s="23"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="15"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1693,19 +1657,15 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="21">
-        <v>45999</v>
-      </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="23"/>
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="14"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
       <c r="E19" s="10"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="15"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1742,18 +1702,14 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B20" s="21">
-        <v>45988</v>
-      </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="11"/>
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="14"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="13"/>
       <c r="E20" s="10"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
       <c r="H20" s="15"/>
       <c r="I20"/>
       <c r="J20"/>
@@ -1791,19 +1747,7 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B21" s="21">
-        <v>46083</v>
-      </c>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="23"/>
-      <c r="H21" s="15"/>
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1840,15 +1784,7 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="14"/>
-      <c r="B22" s="21"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="15"/>
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -1876,16 +1812,8 @@
       <c r="AG22"/>
       <c r="AH22"/>
       <c r="AI22"/>
-      <c r="AJ22"/>
-      <c r="AK22"/>
-      <c r="AL22"/>
-      <c r="AM22"/>
-      <c r="AN22"/>
-      <c r="AO22"/>
-      <c r="AP22"/>
-      <c r="AQ22"/>
-    </row>
-    <row r="23" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -1922,7 +1850,7 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.299999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -1950,8 +1878,16 @@
       <c r="AG24"/>
       <c r="AH24"/>
       <c r="AI24"/>
-    </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AJ24"/>
+      <c r="AK24"/>
+      <c r="AL24"/>
+      <c r="AM24"/>
+      <c r="AN24"/>
+      <c r="AO24"/>
+      <c r="AP24"/>
+      <c r="AQ24"/>
+    </row>
+    <row r="25" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -1988,7 +1924,7 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.4" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2025,7 +1961,7 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2062,7 +1998,7 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2099,7 +2035,15 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29"/>
+      <c r="B29"/>
+      <c r="C29"/>
+      <c r="D29"/>
+      <c r="E29"/>
+      <c r="F29"/>
+      <c r="G29"/>
+      <c r="H29"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2136,7 +2080,15 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30"/>
+      <c r="B30"/>
+      <c r="C30"/>
+      <c r="D30"/>
+      <c r="E30"/>
+      <c r="F30"/>
+      <c r="G30"/>
+      <c r="H30"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2173,7 +2125,7 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:43" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31"/>
       <c r="B31"/>
       <c r="C31"/>
@@ -2218,7 +2170,7 @@
       <c r="AP31"/>
       <c r="AQ31"/>
     </row>
-    <row r="32" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32"/>
       <c r="B32"/>
       <c r="C32"/>
@@ -2263,7 +2215,7 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33"/>
       <c r="B33"/>
       <c r="C33"/>
@@ -2308,7 +2260,7 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34"/>
       <c r="B34"/>
       <c r="C34"/>
@@ -2353,7 +2305,7 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35"/>
       <c r="B35"/>
       <c r="C35"/>
@@ -2398,7 +2350,7 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36"/>
       <c r="B36"/>
       <c r="C36"/>
@@ -2443,7 +2395,7 @@
       <c r="AP36"/>
       <c r="AQ36"/>
     </row>
-    <row r="37" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37"/>
       <c r="B37"/>
       <c r="C37"/>
@@ -2488,7 +2440,7 @@
       <c r="AP37"/>
       <c r="AQ37"/>
     </row>
-    <row r="38" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38"/>
       <c r="B38"/>
       <c r="C38"/>
@@ -2533,133 +2485,63 @@
       <c r="AP38"/>
       <c r="AQ38"/>
     </row>
-    <row r="39" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39"/>
-      <c r="B39"/>
-      <c r="C39"/>
-      <c r="D39"/>
-      <c r="E39"/>
-      <c r="F39"/>
-      <c r="G39"/>
-      <c r="H39"/>
-      <c r="I39"/>
-      <c r="J39"/>
-      <c r="K39"/>
-      <c r="L39"/>
-      <c r="M39"/>
-      <c r="N39"/>
-      <c r="O39"/>
-      <c r="P39"/>
-      <c r="Q39"/>
-      <c r="R39"/>
-      <c r="S39"/>
-      <c r="T39"/>
-      <c r="U39"/>
-      <c r="V39"/>
-      <c r="W39"/>
-      <c r="X39"/>
-      <c r="Y39"/>
-      <c r="Z39"/>
-      <c r="AA39"/>
-      <c r="AB39"/>
-      <c r="AC39"/>
-      <c r="AD39"/>
-      <c r="AE39"/>
-      <c r="AF39"/>
-      <c r="AG39"/>
-      <c r="AH39"/>
-      <c r="AI39"/>
-      <c r="AJ39"/>
-      <c r="AK39"/>
-      <c r="AL39"/>
-      <c r="AM39"/>
-      <c r="AN39"/>
-      <c r="AO39"/>
-      <c r="AP39"/>
-      <c r="AQ39"/>
-    </row>
-    <row r="40" spans="1:43" s="12" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40"/>
-      <c r="B40"/>
-      <c r="C40"/>
-      <c r="D40"/>
-      <c r="E40"/>
-      <c r="F40"/>
-      <c r="G40"/>
-      <c r="H40"/>
-      <c r="I40"/>
-      <c r="J40"/>
-      <c r="K40"/>
-      <c r="L40"/>
-      <c r="M40"/>
-      <c r="N40"/>
-      <c r="O40"/>
-      <c r="P40"/>
-      <c r="Q40"/>
-      <c r="R40"/>
-      <c r="S40"/>
-      <c r="T40"/>
-      <c r="U40"/>
-      <c r="V40"/>
-      <c r="W40"/>
-      <c r="X40"/>
-      <c r="Y40"/>
-      <c r="Z40"/>
-      <c r="AA40"/>
-      <c r="AB40"/>
-      <c r="AC40"/>
-      <c r="AD40"/>
-      <c r="AE40"/>
-      <c r="AF40"/>
-      <c r="AG40"/>
-      <c r="AH40"/>
-      <c r="AI40"/>
-      <c r="AJ40"/>
-      <c r="AK40"/>
-      <c r="AL40"/>
-      <c r="AM40"/>
-      <c r="AN40"/>
-      <c r="AO40"/>
-      <c r="AP40"/>
-      <c r="AQ40"/>
-    </row>
-    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="49" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="50" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="51" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="52" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="53" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="54" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="55" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="56" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="57" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="58" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="59" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="60" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="61" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="62" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="63" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="64" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="65" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="66" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="67" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="68" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="69" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="70" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="71" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="72" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="73" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="74" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="75" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="76" spans="1:8" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="77" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="62" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="63" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="1"/>
+      <c r="B75" s="1"/>
+      <c r="C75" s="1"/>
+      <c r="D75" s="1"/>
+      <c r="E75" s="1"/>
+      <c r="F75" s="1"/>
+      <c r="G75" s="1"/>
+      <c r="H75" s="1"/>
+    </row>
+    <row r="76" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="1"/>
+      <c r="B76" s="1"/>
+      <c r="C76" s="1"/>
+      <c r="D76" s="1"/>
+      <c r="E76" s="1"/>
+      <c r="F76" s="1"/>
+      <c r="G76" s="1"/>
+      <c r="H76" s="1"/>
+    </row>
+    <row r="77" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
@@ -2669,7 +2551,7 @@
       <c r="G77" s="1"/>
       <c r="H77" s="1"/>
     </row>
-    <row r="78" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
@@ -2679,7 +2561,7 @@
       <c r="G78" s="1"/>
       <c r="H78" s="1"/>
     </row>
-    <row r="79" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -2689,7 +2571,7 @@
       <c r="G79" s="1"/>
       <c r="H79" s="1"/>
     </row>
-    <row r="80" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
@@ -2699,7 +2581,7 @@
       <c r="G80" s="1"/>
       <c r="H80" s="1"/>
     </row>
-    <row r="81" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
@@ -2709,7 +2591,7 @@
       <c r="G81" s="1"/>
       <c r="H81" s="1"/>
     </row>
-    <row r="82" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -2719,7 +2601,7 @@
       <c r="G82" s="1"/>
       <c r="H82" s="1"/>
     </row>
-    <row r="83" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -2729,7 +2611,7 @@
       <c r="G83" s="1"/>
       <c r="H83" s="1"/>
     </row>
-    <row r="84" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -2739,31 +2621,11 @@
       <c r="G84" s="1"/>
       <c r="H84" s="1"/>
     </row>
-    <row r="85" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="1"/>
-      <c r="B85" s="1"/>
-      <c r="C85" s="1"/>
-      <c r="D85" s="1"/>
-      <c r="E85" s="1"/>
-      <c r="F85" s="1"/>
-      <c r="G85" s="1"/>
-      <c r="H85" s="1"/>
-    </row>
-    <row r="86" spans="1:8" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="1"/>
-      <c r="B86" s="1"/>
-      <c r="C86" s="1"/>
-      <c r="D86" s="1"/>
-      <c r="E86" s="1"/>
-      <c r="F86" s="1"/>
-      <c r="G86" s="1"/>
-      <c r="H86" s="1"/>
-    </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
@@ -2782,21 +2644,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE61FC198FD4E04C96E2911297C841B3" ma:contentTypeVersion="8" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="0b959ec108c34df947939bcafe18ca0f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2ff38d6f-fd02-4fdf-92f9-9e1de7e56b4e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ea491a5a738f7edb69f4b3365f69f6f5" ns2:_="">
     <xsd:import namespace="2ff38d6f-fd02-4fdf-92f9-9e1de7e56b4e"/>
@@ -2964,24 +2811,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11A7DB11-1CAE-4437-8A7A-AB5070F8CF2F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E7CCC5C-68BB-462F-8DF9-8CB8E30B9C1A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAB071C6-73BD-41AC-BC6C-528FC4CACB9B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2997,4 +2842,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E7CCC5C-68BB-462F-8DF9-8CB8E30B9C1A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11A7DB11-1CAE-4437-8A7A-AB5070F8CF2F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Mise à jour du tableau de compétences E5
</commit_message>
<xml_diff>
--- a/e5/tableau_competences.xlsx
+++ b/e5/tableau_competences.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e2f25182b63ad68a/Documents/PORTEFOLIO/e5/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mon Drive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4AF58D0-E6C5-40B8-A23E-99B808EF88C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{828886A8-79CC-4F6C-A0CE-02E5C30AF230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$22</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -160,6 +160,30 @@
   <si>
     <t>Développement de l'employabilité et du réseau via Linkedin</t>
   </si>
+  <si>
+    <t>Simulation d'une infrastructure réseau d'entreprise avec segmentation VLAN, firewall pfSense et Active Directory</t>
+  </si>
+  <si>
+    <t>Procédure dotation d'un nouveau PC</t>
+  </si>
+  <si>
+    <t>Projet Etherchannel HSRP</t>
+  </si>
+  <si>
+    <t>Gestion et suivi de la cession de matériel informatique usagé au personnel de Quick France</t>
+  </si>
+  <si>
+    <t>Création et configuration de badges utilisateurs sur le logiciel Optimidoc</t>
+  </si>
+  <si>
+    <t>Réinitialisation et remise en état des postes informatiques lors des départs de collaborateurs</t>
+  </si>
+  <si>
+    <t>Préparation et configuration des postes informatiques pour les nouveaux collaborateurs</t>
+  </si>
+  <si>
+    <t>05/06/52025</t>
+  </si>
 </sst>
 </file>
 
@@ -168,7 +192,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -238,6 +262,12 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -522,7 +552,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -560,9 +590,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -601,6 +628,27 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -968,7 +1016,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ84"/>
+  <dimension ref="A1:AQ86"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
@@ -979,58 +1027,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="38"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
     </row>
     <row r="3" spans="1:43" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="18"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="17"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="41"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
       <c r="F4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="24" t="s">
+      <c r="G4" s="23" t="s">
         <v>4</v>
       </c>
       <c r="H4" s="7" t="s">
@@ -1038,22 +1086,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="44" t="s">
+      <c r="A5" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="45"/>
+      <c r="B5" s="51"/>
+      <c r="C5" s="51"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="51"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="51"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="42" t="s">
+      <c r="A6" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="42" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -1076,24 +1124,24 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="43"/>
-      <c r="B7" s="37"/>
-      <c r="C7" s="19" t="s">
+      <c r="A7" s="49"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="20" t="s">
+      <c r="H7" s="19" t="s">
         <v>19</v>
       </c>
       <c r="I7"/>
@@ -1133,16 +1181,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="29"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="35"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1183,7 +1231,7 @@
       <c r="A9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="20">
         <v>45993</v>
       </c>
       <c r="C9" s="11"/>
@@ -1232,7 +1280,7 @@
       <c r="A10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="21">
+      <c r="B10" s="20">
         <v>45998</v>
       </c>
       <c r="C10" s="11"/>
@@ -1281,7 +1329,7 @@
       <c r="A11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="21">
+      <c r="B11" s="20">
         <v>45978</v>
       </c>
       <c r="C11" s="10"/>
@@ -1289,7 +1337,7 @@
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
       <c r="G11" s="10"/>
-      <c r="H11" s="25"/>
+      <c r="H11" s="24"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1328,17 +1376,17 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="26"/>
+        <v>33</v>
+      </c>
+      <c r="B12" s="26">
+        <v>46082</v>
+      </c>
+      <c r="C12" s="30"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="29"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1376,16 +1424,18 @@
       <c r="AQ12"/>
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="31"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="31"/>
-      <c r="F13" s="31"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="32"/>
+      <c r="A13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="31">
+        <v>46029</v>
+      </c>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="29"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1423,14 +1473,18 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5"/>
-      <c r="B14" s="21"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
+      <c r="A14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="25"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1468,14 +1522,16 @@
       <c r="AQ14"/>
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
+      <c r="A15" s="36" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="38"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1513,16 +1569,18 @@
       <c r="AQ15"/>
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="35"/>
+      <c r="A16" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="20">
+        <v>45813</v>
+      </c>
+      <c r="C16" s="10"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="10"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1560,17 +1618,17 @@
       <c r="AQ16"/>
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" s="21">
-        <v>45999</v>
-      </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="23"/>
+      <c r="A17" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="22"/>
+      <c r="D17" s="11"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="10"/>
       <c r="H17" s="10"/>
       <c r="I17"/>
       <c r="J17"/>
@@ -1609,18 +1667,16 @@
       <c r="AQ17"/>
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="21">
-        <v>45988</v>
-      </c>
-      <c r="C18" s="23"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="15"/>
+      <c r="A18" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="40"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="41"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1658,14 +1714,18 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="14"/>
-      <c r="B19" s="21"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
+      <c r="A19" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="20">
+        <v>45999</v>
+      </c>
+      <c r="C19" s="11"/>
+      <c r="D19" s="22"/>
       <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="15"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="10"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1703,14 +1763,18 @@
       <c r="AQ19"/>
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="14"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="13"/>
+      <c r="A20" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="20">
+        <v>45988</v>
+      </c>
+      <c r="C20" s="22"/>
+      <c r="D20" s="11"/>
       <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="15"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="14"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1748,6 +1812,18 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="20">
+        <v>46083</v>
+      </c>
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="14"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1785,6 +1861,18 @@
       <c r="AQ21"/>
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="20">
+        <v>46128</v>
+      </c>
+      <c r="C22" s="11"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="14"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -1812,8 +1900,28 @@
       <c r="AG22"/>
       <c r="AH22"/>
       <c r="AI22"/>
+      <c r="AJ22"/>
+      <c r="AK22"/>
+      <c r="AL22"/>
+      <c r="AM22"/>
+      <c r="AN22"/>
+      <c r="AO22"/>
+      <c r="AP22"/>
+      <c r="AQ22"/>
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="20">
+        <v>46114</v>
+      </c>
+      <c r="C23" s="10"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="14"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -1850,7 +1958,7 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.299999999999997" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -1878,16 +1986,8 @@
       <c r="AG24"/>
       <c r="AH24"/>
       <c r="AI24"/>
-      <c r="AJ24"/>
-      <c r="AK24"/>
-      <c r="AL24"/>
-      <c r="AM24"/>
-      <c r="AN24"/>
-      <c r="AO24"/>
-      <c r="AP24"/>
-      <c r="AQ24"/>
-    </row>
-    <row r="25" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -1924,7 +2024,7 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2036,14 +2136,6 @@
       <c r="AQ28"/>
     </row>
     <row r="29" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29"/>
-      <c r="B29"/>
-      <c r="C29"/>
-      <c r="D29"/>
-      <c r="E29"/>
-      <c r="F29"/>
-      <c r="G29"/>
-      <c r="H29"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2081,14 +2173,6 @@
       <c r="AQ29"/>
     </row>
     <row r="30" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30"/>
-      <c r="B30"/>
-      <c r="C30"/>
-      <c r="D30"/>
-      <c r="E30"/>
-      <c r="F30"/>
-      <c r="G30"/>
-      <c r="H30"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2125,7 +2209,7 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31"/>
       <c r="B31"/>
       <c r="C31"/>
@@ -2215,7 +2299,7 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:43" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33"/>
       <c r="B33"/>
       <c r="C33"/>
@@ -2485,8 +2569,96 @@
       <c r="AP38"/>
       <c r="AQ38"/>
     </row>
-    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39"/>
+      <c r="B39"/>
+      <c r="C39"/>
+      <c r="D39"/>
+      <c r="E39"/>
+      <c r="F39"/>
+      <c r="G39"/>
+      <c r="H39"/>
+      <c r="I39"/>
+      <c r="J39"/>
+      <c r="K39"/>
+      <c r="L39"/>
+      <c r="M39"/>
+      <c r="N39"/>
+      <c r="O39"/>
+      <c r="P39"/>
+      <c r="Q39"/>
+      <c r="R39"/>
+      <c r="S39"/>
+      <c r="T39"/>
+      <c r="U39"/>
+      <c r="V39"/>
+      <c r="W39"/>
+      <c r="X39"/>
+      <c r="Y39"/>
+      <c r="Z39"/>
+      <c r="AA39"/>
+      <c r="AB39"/>
+      <c r="AC39"/>
+      <c r="AD39"/>
+      <c r="AE39"/>
+      <c r="AF39"/>
+      <c r="AG39"/>
+      <c r="AH39"/>
+      <c r="AI39"/>
+      <c r="AJ39"/>
+      <c r="AK39"/>
+      <c r="AL39"/>
+      <c r="AM39"/>
+      <c r="AN39"/>
+      <c r="AO39"/>
+      <c r="AP39"/>
+      <c r="AQ39"/>
+    </row>
+    <row r="40" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40"/>
+      <c r="B40"/>
+      <c r="C40"/>
+      <c r="D40"/>
+      <c r="E40"/>
+      <c r="F40"/>
+      <c r="G40"/>
+      <c r="H40"/>
+      <c r="I40"/>
+      <c r="J40"/>
+      <c r="K40"/>
+      <c r="L40"/>
+      <c r="M40"/>
+      <c r="N40"/>
+      <c r="O40"/>
+      <c r="P40"/>
+      <c r="Q40"/>
+      <c r="R40"/>
+      <c r="S40"/>
+      <c r="T40"/>
+      <c r="U40"/>
+      <c r="V40"/>
+      <c r="W40"/>
+      <c r="X40"/>
+      <c r="Y40"/>
+      <c r="Z40"/>
+      <c r="AA40"/>
+      <c r="AB40"/>
+      <c r="AC40"/>
+      <c r="AD40"/>
+      <c r="AE40"/>
+      <c r="AF40"/>
+      <c r="AG40"/>
+      <c r="AH40"/>
+      <c r="AI40"/>
+      <c r="AJ40"/>
+      <c r="AK40"/>
+      <c r="AL40"/>
+      <c r="AM40"/>
+      <c r="AN40"/>
+      <c r="AO40"/>
+      <c r="AP40"/>
+      <c r="AQ40"/>
+    </row>
     <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -2521,26 +2693,8 @@
     <row r="72" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="73" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="74" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="1"/>
-      <c r="B75" s="1"/>
-      <c r="C75" s="1"/>
-      <c r="D75" s="1"/>
-      <c r="E75" s="1"/>
-      <c r="F75" s="1"/>
-      <c r="G75" s="1"/>
-      <c r="H75" s="1"/>
-    </row>
-    <row r="76" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="1"/>
-      <c r="B76" s="1"/>
-      <c r="C76" s="1"/>
-      <c r="D76" s="1"/>
-      <c r="E76" s="1"/>
-      <c r="F76" s="1"/>
-      <c r="G76" s="1"/>
-      <c r="H76" s="1"/>
-    </row>
+    <row r="75" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="77" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
@@ -2621,11 +2775,31 @@
       <c r="G84" s="1"/>
       <c r="H84" s="1"/>
     </row>
+    <row r="85" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="1"/>
+      <c r="B85" s="1"/>
+      <c r="C85" s="1"/>
+      <c r="D85" s="1"/>
+      <c r="E85" s="1"/>
+      <c r="F85" s="1"/>
+      <c r="G85" s="1"/>
+      <c r="H85" s="1"/>
+    </row>
+    <row r="86" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="1"/>
+      <c r="B86" s="1"/>
+      <c r="C86" s="1"/>
+      <c r="D86" s="1"/>
+      <c r="E86" s="1"/>
+      <c r="F86" s="1"/>
+      <c r="G86" s="1"/>
+      <c r="H86" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
@@ -2644,6 +2818,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE61FC198FD4E04C96E2911297C841B3" ma:contentTypeVersion="8" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="0b959ec108c34df947939bcafe18ca0f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2ff38d6f-fd02-4fdf-92f9-9e1de7e56b4e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ea491a5a738f7edb69f4b3365f69f6f5" ns2:_="">
     <xsd:import namespace="2ff38d6f-fd02-4fdf-92f9-9e1de7e56b4e"/>
@@ -2811,22 +3000,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E7CCC5C-68BB-462F-8DF9-8CB8E30B9C1A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11A7DB11-1CAE-4437-8A7A-AB5070F8CF2F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAB071C6-73BD-41AC-BC6C-528FC4CACB9B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2842,21 +3033,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E7CCC5C-68BB-462F-8DF9-8CB8E30B9C1A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11A7DB11-1CAE-4437-8A7A-AB5070F8CF2F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Ajout du projet GLPI et mise à jour du tableau de compétences
</commit_message>
<xml_diff>
--- a/e5/tableau_competences.xlsx
+++ b/e5/tableau_competences.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mon Drive\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mirim\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{828886A8-79CC-4F6C-A0CE-02E5C30AF230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D423031-C14A-4F63-B22B-C05C02CEBEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$24</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="43">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -152,9 +152,6 @@
     <t>Création de mon Portfolio</t>
   </si>
   <si>
-    <t xml:space="preserve">         13/12/2025</t>
-  </si>
-  <si>
     <t>Adresse URL du portfolio : https://miri94400.github.io/PortefolioMiri/</t>
   </si>
   <si>
@@ -182,7 +179,16 @@
     <t>Préparation et configuration des postes informatiques pour les nouveaux collaborateurs</t>
   </si>
   <si>
-    <t>05/06/52025</t>
+    <t>Mise en place de GLPI avec synchronisation Active Directory et gestion de tickets StadiumCompany</t>
+  </si>
+  <si>
+    <t>2025/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         2025/2026</t>
+  </si>
+  <si>
+    <t>Configuration de PC</t>
   </si>
 </sst>
 </file>
@@ -552,7 +558,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -706,6 +712,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1016,7 +1028,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ86"/>
+  <dimension ref="A1:AQ88"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
@@ -1087,7 +1099,7 @@
     </row>
     <row r="5" spans="1:43" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="50" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" s="51"/>
       <c r="C5" s="51"/>
@@ -1231,8 +1243,8 @@
       <c r="A9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="20">
-        <v>45993</v>
+      <c r="B9" s="20" t="s">
+        <v>40</v>
       </c>
       <c r="C9" s="11"/>
       <c r="D9" s="8"/>
@@ -1280,8 +1292,8 @@
       <c r="A10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="20">
-        <v>45998</v>
+      <c r="B10" s="20" t="s">
+        <v>40</v>
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
@@ -1327,10 +1339,10 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="20">
-        <v>45978</v>
+        <v>31</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>40</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="8"/>
@@ -1376,10 +1388,10 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="26">
-        <v>46082</v>
+        <v>32</v>
+      </c>
+      <c r="B12" s="26" t="s">
+        <v>40</v>
       </c>
       <c r="C12" s="30"/>
       <c r="D12" s="32"/>
@@ -1425,10 +1437,10 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="31">
-        <v>46029</v>
+        <v>34</v>
+      </c>
+      <c r="B13" s="31" t="s">
+        <v>40</v>
       </c>
       <c r="C13" s="30"/>
       <c r="D13" s="30"/>
@@ -1474,17 +1486,17 @@
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="25"/>
+        <v>39</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="29"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1522,16 +1534,18 @@
       <c r="AQ14"/>
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="38"/>
+      <c r="A15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="25"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1569,18 +1583,16 @@
       <c r="AQ15"/>
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" s="20">
-        <v>45813</v>
-      </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="10"/>
+      <c r="A16" s="36" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="38"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1624,11 +1636,11 @@
       <c r="B17" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="11"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="22"/>
       <c r="E17" s="10"/>
       <c r="F17" s="11"/>
-      <c r="G17" s="10"/>
+      <c r="G17" s="11"/>
       <c r="H17" s="10"/>
       <c r="I17"/>
       <c r="J17"/>
@@ -1667,16 +1679,18 @@
       <c r="AQ17"/>
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="39" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="41"/>
+      <c r="A18" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="22"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1714,18 +1728,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="20">
-        <v>45999</v>
-      </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="10"/>
+      <c r="A19" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="40"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="40"/>
+      <c r="F19" s="40"/>
+      <c r="G19" s="40"/>
+      <c r="H19" s="41"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1763,18 +1775,18 @@
       <c r="AQ19"/>
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B20" s="20">
-        <v>45988</v>
-      </c>
-      <c r="C20" s="22"/>
-      <c r="D20" s="11"/>
+      <c r="A20" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="11"/>
+      <c r="D20" s="22"/>
       <c r="E20" s="10"/>
-      <c r="F20" s="11"/>
+      <c r="F20" s="22"/>
       <c r="G20" s="11"/>
-      <c r="H20" s="14"/>
+      <c r="H20" s="10"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1812,18 +1824,16 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="B21" s="20">
-        <v>46083</v>
-      </c>
-      <c r="C21" s="22"/>
+      <c r="A21" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="20"/>
+      <c r="C21" s="11"/>
       <c r="D21" s="22"/>
       <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="14"/>
+      <c r="F21" s="53"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="52"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1862,16 +1872,16 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="B22" s="20">
-        <v>46128</v>
-      </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="22"/>
+        <v>27</v>
+      </c>
+      <c r="B22" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="22"/>
+      <c r="D22" s="11"/>
       <c r="E22" s="10"/>
       <c r="F22" s="11"/>
-      <c r="G22" s="10"/>
+      <c r="G22" s="11"/>
       <c r="H22" s="14"/>
       <c r="I22"/>
       <c r="J22"/>
@@ -1911,16 +1921,16 @@
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="B23" s="20">
-        <v>46114</v>
-      </c>
-      <c r="C23" s="10"/>
+        <v>33</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C23" s="22"/>
       <c r="D23" s="22"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
-      <c r="G23" s="11"/>
+      <c r="G23" s="22"/>
       <c r="H23" s="14"/>
       <c r="I23"/>
       <c r="J23"/>
@@ -1959,6 +1969,18 @@
       <c r="AQ23"/>
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="11"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="14"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -1986,8 +2008,28 @@
       <c r="AG24"/>
       <c r="AH24"/>
       <c r="AI24"/>
+      <c r="AJ24"/>
+      <c r="AK24"/>
+      <c r="AL24"/>
+      <c r="AM24"/>
+      <c r="AN24"/>
+      <c r="AO24"/>
+      <c r="AP24"/>
+      <c r="AQ24"/>
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" s="10"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="14"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2024,7 +2066,7 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2052,16 +2094,8 @@
       <c r="AG26"/>
       <c r="AH26"/>
       <c r="AI26"/>
-      <c r="AJ26"/>
-      <c r="AK26"/>
-      <c r="AL26"/>
-      <c r="AM26"/>
-      <c r="AN26"/>
-      <c r="AO26"/>
-      <c r="AP26"/>
-      <c r="AQ26"/>
-    </row>
-    <row r="27" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2098,7 +2132,7 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2210,14 +2244,6 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31"/>
-      <c r="B31"/>
-      <c r="C31"/>
-      <c r="D31"/>
-      <c r="E31"/>
-      <c r="F31"/>
-      <c r="G31"/>
-      <c r="H31"/>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2255,14 +2281,6 @@
       <c r="AQ31"/>
     </row>
     <row r="32" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32"/>
-      <c r="B32"/>
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32"/>
-      <c r="F32"/>
-      <c r="G32"/>
-      <c r="H32"/>
       <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2299,7 +2317,7 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33"/>
       <c r="B33"/>
       <c r="C33"/>
@@ -2389,7 +2407,7 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:43" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35"/>
       <c r="B35"/>
       <c r="C35"/>
@@ -2659,8 +2677,96 @@
       <c r="AP40"/>
       <c r="AQ40"/>
     </row>
-    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41"/>
+      <c r="B41"/>
+      <c r="C41"/>
+      <c r="D41"/>
+      <c r="E41"/>
+      <c r="F41"/>
+      <c r="G41"/>
+      <c r="H41"/>
+      <c r="I41"/>
+      <c r="J41"/>
+      <c r="K41"/>
+      <c r="L41"/>
+      <c r="M41"/>
+      <c r="N41"/>
+      <c r="O41"/>
+      <c r="P41"/>
+      <c r="Q41"/>
+      <c r="R41"/>
+      <c r="S41"/>
+      <c r="T41"/>
+      <c r="U41"/>
+      <c r="V41"/>
+      <c r="W41"/>
+      <c r="X41"/>
+      <c r="Y41"/>
+      <c r="Z41"/>
+      <c r="AA41"/>
+      <c r="AB41"/>
+      <c r="AC41"/>
+      <c r="AD41"/>
+      <c r="AE41"/>
+      <c r="AF41"/>
+      <c r="AG41"/>
+      <c r="AH41"/>
+      <c r="AI41"/>
+      <c r="AJ41"/>
+      <c r="AK41"/>
+      <c r="AL41"/>
+      <c r="AM41"/>
+      <c r="AN41"/>
+      <c r="AO41"/>
+      <c r="AP41"/>
+      <c r="AQ41"/>
+    </row>
+    <row r="42" spans="1:43" s="12" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42"/>
+      <c r="B42"/>
+      <c r="C42"/>
+      <c r="D42"/>
+      <c r="E42"/>
+      <c r="F42"/>
+      <c r="G42"/>
+      <c r="H42"/>
+      <c r="I42"/>
+      <c r="J42"/>
+      <c r="K42"/>
+      <c r="L42"/>
+      <c r="M42"/>
+      <c r="N42"/>
+      <c r="O42"/>
+      <c r="P42"/>
+      <c r="Q42"/>
+      <c r="R42"/>
+      <c r="S42"/>
+      <c r="T42"/>
+      <c r="U42"/>
+      <c r="V42"/>
+      <c r="W42"/>
+      <c r="X42"/>
+      <c r="Y42"/>
+      <c r="Z42"/>
+      <c r="AA42"/>
+      <c r="AB42"/>
+      <c r="AC42"/>
+      <c r="AD42"/>
+      <c r="AE42"/>
+      <c r="AF42"/>
+      <c r="AG42"/>
+      <c r="AH42"/>
+      <c r="AI42"/>
+      <c r="AJ42"/>
+      <c r="AK42"/>
+      <c r="AL42"/>
+      <c r="AM42"/>
+      <c r="AN42"/>
+      <c r="AO42"/>
+      <c r="AP42"/>
+      <c r="AQ42"/>
+    </row>
     <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -2695,26 +2801,8 @@
     <row r="74" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="75" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="76" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="1"/>
-      <c r="B77" s="1"/>
-      <c r="C77" s="1"/>
-      <c r="D77" s="1"/>
-      <c r="E77" s="1"/>
-      <c r="F77" s="1"/>
-      <c r="G77" s="1"/>
-      <c r="H77" s="1"/>
-    </row>
-    <row r="78" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="1"/>
-      <c r="B78" s="1"/>
-      <c r="C78" s="1"/>
-      <c r="D78" s="1"/>
-      <c r="E78" s="1"/>
-      <c r="F78" s="1"/>
-      <c r="G78" s="1"/>
-      <c r="H78" s="1"/>
-    </row>
+    <row r="77" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="79" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
@@ -2795,11 +2883,31 @@
       <c r="G86" s="1"/>
       <c r="H86" s="1"/>
     </row>
+    <row r="87" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="1"/>
+      <c r="B87" s="1"/>
+      <c r="C87" s="1"/>
+      <c r="D87" s="1"/>
+      <c r="E87" s="1"/>
+      <c r="F87" s="1"/>
+      <c r="G87" s="1"/>
+      <c r="H87" s="1"/>
+    </row>
+    <row r="88" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="1"/>
+      <c r="B88" s="1"/>
+      <c r="C88" s="1"/>
+      <c r="D88" s="1"/>
+      <c r="E88" s="1"/>
+      <c r="F88" s="1"/>
+      <c r="G88" s="1"/>
+      <c r="H88" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
@@ -2818,18 +2926,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3001,18 +3109,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E7CCC5C-68BB-462F-8DF9-8CB8E30B9C1A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11A7DB11-1CAE-4437-8A7A-AB5070F8CF2F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11A7DB11-1CAE-4437-8A7A-AB5070F8CF2F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E7CCC5C-68BB-462F-8DF9-8CB8E30B9C1A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>